<commit_message>
feat: rebuild catalog logic, fix empty categories and sync category tree
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -2716,48 +2716,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>197</xdr:row>
-      <xdr:rowOff>9360</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>-11925360</xdr:colOff>
-      <xdr:row>197</xdr:row>
-      <xdr:rowOff>2199600</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Имя " descr=""/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="129240" y="426332880"/>
-          <a:ext cx="360000" cy="2190240"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
@@ -2770,12 +2728,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="42.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="1" width="63.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="7.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="7.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="3.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="3.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="13" style="0" width="10.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="13" style="0" width="10.44"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="4.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9467,7 +9425,7 @@
         <v>644</v>
       </c>
       <c r="F196" s="9" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="G196" s="9" t="s">
         <v>649</v>
@@ -9503,7 +9461,7 @@
         <v>644</v>
       </c>
       <c r="F197" s="9" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="G197" s="9" t="s">
         <v>653</v>
@@ -9539,7 +9497,7 @@
         <v>644</v>
       </c>
       <c r="F198" s="9" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="G198" s="9" t="s">
         <v>657</v>
@@ -9575,7 +9533,7 @@
         <v>644</v>
       </c>
       <c r="F199" s="9" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="G199" s="9" t="s">
         <v>661</v>
@@ -9611,7 +9569,7 @@
         <v>644</v>
       </c>
       <c r="F200" s="9" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="G200" s="20" t="s">
         <v>661</v>
@@ -10658,6 +10616,5 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>